<commit_message>
Added disponibil pt vanzare field in xls
</commit_message>
<xml_diff>
--- a/src/data/exhibition-imports/template/artist-submission-template.xlsx
+++ b/src/data/exhibition-imports/template/artist-submission-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Study/Projects/Cutare/cutare-gallery/src/data/exhibition-imports/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07EA0879-88D0-4D49-8317-D34A68408122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A7B7D1D-3D02-4D43-BC4B-B976B0FDEB65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,36 +25,26 @@
     <author>Eliza Balica</author>
   </authors>
   <commentList>
-    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{5D19A723-DD33-3E4F-AC47-8E1871DAE85D}">
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{D76744CC-DB04-8D40-B720-9432E2207477}">
       <text>
         <r>
           <rPr>
             <b/>
-            <sz val="10"/>
+            <sz val="16"/>
             <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
+            <rFont val="Calibri"/>
             <family val="2"/>
           </rPr>
-          <t>Se completeaza de catre curator</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
+          <t>Se completează de către curator</t>
         </r>
       </text>
     </comment>
-    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{EC8AFA6F-DF5D-BC40-BE74-A8E77B827617}">
+    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{EC8AFA6F-DF5D-BC40-BE74-A8E77B827617}">
       <text>
         <r>
           <rPr>
             <b/>
-            <sz val="14"/>
+            <sz val="16"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
             <family val="2"/>
@@ -63,7 +53,7 @@
         </r>
         <r>
           <rPr>
-            <sz val="14"/>
+            <sz val="16"/>
             <color rgb="FF000000"/>
             <rFont val="Calibri"/>
             <family val="2"/>
@@ -78,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="11">
   <si>
     <t>nume artist</t>
   </si>
@@ -108,13 +98,16 @@
   </si>
   <si>
     <t>sala</t>
+  </si>
+  <si>
+    <t>disponibila pentru vanzare (da/nu)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -135,27 +128,14 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
+      <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -249,7 +229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -277,6 +257,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -620,18 +603,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="24" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="39.83203125" style="2" customWidth="1"/>
     <col min="2" max="2" width="20" style="1" customWidth="1"/>
     <col min="3" max="3" width="60" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.1640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.1640625" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.83203125" style="1"/>
+    <col min="4" max="4" width="48.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.1640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -639,8 +623,9 @@
       <c r="C1" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D1" s="11"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>2</v>
       </c>
@@ -650,8 +635,9 @@
       <c r="C2" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D2" s="11"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>3</v>
       </c>
@@ -661,8 +647,9 @@
       <c r="C3" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D3" s="11"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>4</v>
       </c>
@@ -672,10 +659,11 @@
       <c r="C4" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D4" s="11"/>
+    </row>
+    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>5</v>
       </c>
@@ -686,13 +674,16 @@
         <v>7</v>
       </c>
       <c r="D7" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="F7" s="7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>1</v>
       </c>
@@ -702,14 +693,15 @@
       <c r="C8" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>1</v>
-      </c>
+      <c r="D8" s="6"/>
       <c r="E8" s="6" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F8" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>1</v>
       </c>
@@ -719,14 +711,15 @@
       <c r="C9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F9" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>1</v>
       </c>
@@ -736,14 +729,15 @@
       <c r="C10" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F10" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>1</v>
       </c>
@@ -753,14 +747,15 @@
       <c r="C11" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F11" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>1</v>
       </c>
@@ -770,14 +765,15 @@
       <c r="C12" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D12" s="4"/>
       <c r="E12" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F12" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>1</v>
       </c>
@@ -787,14 +783,15 @@
       <c r="C13" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D13" s="4"/>
       <c r="E13" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F13" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>1</v>
       </c>
@@ -804,14 +801,15 @@
       <c r="C14" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D14" s="4"/>
       <c r="E14" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F14" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>1</v>
       </c>
@@ -821,14 +819,15 @@
       <c r="C15" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F15" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>1</v>
       </c>
@@ -838,14 +837,15 @@
       <c r="C16" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F16" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>1</v>
       </c>
@@ -855,10 +855,11 @@
       <c r="C17" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>1</v>
-      </c>
+      <c r="D17" s="4"/>
       <c r="E17" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>